<commit_message>
sign-out required and not required feature and change in import feature and template
</commit_message>
<xml_diff>
--- a/sample_bulk_upload.xlsx
+++ b/sample_bulk_upload.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Participants" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participants" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -450,35 +450,40 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Speciality</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Contact No.</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>WhatsApp Number</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Place of Work</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Institution/Hospital</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Medical License No.</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Participant Type</t>
         </is>
@@ -495,33 +500,32 @@
           <t>Medical Officer</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>ajay.varma100@example.com</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>9751028618</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>9751028618</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Aster Medcity, Kochi</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>TCMC-78494</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -538,33 +542,32 @@
           <t>Nursing Supervisor</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>nikhil.bhat101@example.com</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>9508427798</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>9419280490</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Apollo Hospitals, Chennai</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>TCMC-66207</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -581,33 +584,32 @@
           <t>Medical Officer</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>ananya.varma102@example.com</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>9427899537</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>9427899537</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Apollo Hospitals, Chennai</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>TCMC-23006</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -624,33 +626,32 @@
           <t>Assistant Professor</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>suresh.kurian103@example.com</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>9918982730</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>9918982730</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>KIMS Health, Trivandrum</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>TCMC-96563</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -667,33 +668,32 @@
           <t>Junior Resident</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>divya.krishnan104@example.com</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>9187174381</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>9187174381</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>St. John's Medical College, Bengaluru</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>TCMC-19838</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -710,37 +710,37 @@
           <t>Consultant Physician</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>sara.kurian105@example.com</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>9268075622</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>9268075622</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Apollo Hospitals, Chennai</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>TCMC-71592</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Faculty</t>
         </is>
@@ -757,33 +757,32 @@
           <t>Consultant Physician</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>sneha.varma106@example.com</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>9412737284</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>9412737284</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>KIMS Health, Trivandrum</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>TCMC-69510</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -800,33 +799,32 @@
           <t>Postgraduate Student</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>varun.iyer107@example.com</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>9176428684</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>9176428684</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>KIMS Health, Trivandrum</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>TCMC-91927</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -843,33 +841,32 @@
           <t>Postgraduate Student</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>varun.patel108@example.com</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>9733281747</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>9312406764</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Jubilee Mission Hospital, Thrissur</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>TCMC-25043</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -886,33 +883,32 @@
           <t>Assistant Professor</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>manoj.kumar109@example.com</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>9684719405</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>9684719405</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>KIMS Health, Trivandrum</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>TCMC-28643</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -929,33 +925,32 @@
           <t>Consultant Physician</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>nandini.krishnan110@example.com</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>9176675731</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>9176675731</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>KIMS Health, Trivandrum</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>TCMC-87993</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -972,33 +967,32 @@
           <t>Medical Officer</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>arjun.kurian111@example.com</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>9904187231</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>9571537429</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Government Medical College, Thrissur</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>TCMC-71433</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -1015,33 +1009,32 @@
           <t>Senior Resident</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>karthik.mathew1@example.com</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>9996478772</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>9996478772</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>St. John's Medical College, Bengaluru</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>TCMC-16826</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -1058,29 +1051,27 @@
           <t>Associate Professor</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>anjali.kurian112@example.com</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>9839462365</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>KIMS Health, Trivandrum</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>TCMC-75597</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -1097,33 +1088,32 @@
           <t>Nursing Supervisor</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>divya.nair113@example.com</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>9679800791</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>9679800791</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Apollo Hospitals, Chennai</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>TCMC-15224</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>Speaker</t>
         </is>
@@ -1140,29 +1130,27 @@
           <t>Consultant Surgeon</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>riya.iyer114@example.com</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>9563887247</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>9563887247</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>KIMS Health, Trivandrum</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>delegate</t>
         </is>
@@ -1179,33 +1167,32 @@
           <t>Assistant Professor</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>AJAY.VARMA100@EXAMPLE.COM</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>9198061499</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>9997603725</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Apollo Hospitals, Chennai</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>TCMC-86955</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>Delegate</t>
         </is>
@@ -1222,33 +1209,32 @@
           <t>Staff Nurse</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>divya.patel0@example.com</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>9917364173</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>9917364173</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Jubilee Mission Hospital, Thrissur</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>TCMC-43065</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>Faculty</t>
         </is>

</xml_diff>